<commit_message>
Queue/capacity workbook: numbers-only validation on inputs, checks for text inputs and Variables errors
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013JwSYm4UV7vKHqaUukbU1G
</commit_message>
<xml_diff>
--- a/docs/Queue_Capacity_LoadBalancing.xlsx
+++ b/docs/Queue_Capacity_LoadBalancing.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3212" uniqueCount="561">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3214" uniqueCount="563">
   <si>
     <t xml:space="preserve">Smart Mess: queues, capacity and load balancing</t>
   </si>
@@ -1717,6 +1717,12 @@
   </si>
   <si>
     <t xml:space="preserve">Dynamic routing beats a fixed share at the same compliance on the average day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every input on the Assumptions tab is a number (text such as '12-15' breaks the formulas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No formula errors in Variables</t>
   </si>
   <si>
     <t xml:space="preserve">Takeaway: Over a whole lunch, Σ(time-average people inside × 10 min) = Σ(arrivals × visit time) exactly; the check allows 10% because students who arrive late in a slot spill their minutes into the next one and the run ends when the last student has a seat.</t>
@@ -3527,11 +3533,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="43524926"/>
-        <c:axId val="49962030"/>
+        <c:axId val="71035927"/>
+        <c:axId val="48697126"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="43524926"/>
+        <c:axId val="71035927"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3563,7 +3569,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="49962030"/>
+        <c:crossAx val="48697126"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3571,7 +3577,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="49962030"/>
+        <c:axId val="48697126"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3647,7 +3653,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="43524926"/>
+        <c:crossAx val="71035927"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4652,11 +4658,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="86985046"/>
-        <c:axId val="51984681"/>
+        <c:axId val="69896877"/>
+        <c:axId val="14117920"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="86985046"/>
+        <c:axId val="69896877"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4688,7 +4694,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="51984681"/>
+        <c:crossAx val="14117920"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4696,7 +4702,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="51984681"/>
+        <c:axId val="14117920"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4772,7 +4778,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86985046"/>
+        <c:crossAx val="69896877"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5236,11 +5242,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="38385453"/>
-        <c:axId val="2577831"/>
+        <c:axId val="24799640"/>
+        <c:axId val="81653122"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="38385453"/>
+        <c:axId val="24799640"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5272,7 +5278,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2577831"/>
+        <c:crossAx val="81653122"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5280,7 +5286,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2577831"/>
+        <c:axId val="81653122"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5356,7 +5362,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="38385453"/>
+        <c:crossAx val="24799640"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5627,11 +5633,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="87423132"/>
-        <c:axId val="84478833"/>
+        <c:axId val="32181564"/>
+        <c:axId val="67744161"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="87423132"/>
+        <c:axId val="32181564"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5663,7 +5669,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84478833"/>
+        <c:crossAx val="67744161"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5671,7 +5677,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="84478833"/>
+        <c:axId val="67744161"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5747,7 +5753,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87423132"/>
+        <c:crossAx val="32181564"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5968,11 +5974,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="35462890"/>
-        <c:axId val="93708794"/>
+        <c:axId val="38965680"/>
+        <c:axId val="37597058"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="35462890"/>
+        <c:axId val="38965680"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6004,7 +6010,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93708794"/>
+        <c:crossAx val="37597058"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6012,7 +6018,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="93708794"/>
+        <c:axId val="37597058"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6054,7 +6060,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="35462890"/>
+        <c:crossAx val="38965680"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7034,11 +7040,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="45490891"/>
-        <c:axId val="20776379"/>
+        <c:axId val="13982800"/>
+        <c:axId val="71843819"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="45490891"/>
+        <c:axId val="13982800"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7070,7 +7076,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="20776379"/>
+        <c:crossAx val="71843819"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7078,7 +7084,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="20776379"/>
+        <c:axId val="71843819"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7154,7 +7160,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="45490891"/>
+        <c:crossAx val="13982800"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7838,7 +7844,7 @@
         <v>46</v>
       </c>
       <c r="C28" s="11" t="str">
-        <f aca="false">Checks!C14</f>
+        <f aca="false">Checks!C16</f>
         <v>ALL OK</v>
       </c>
       <c r="D28" s="11"/>
@@ -18553,7 +18559,7 @@
     <tabColor rgb="FFA5A5A5"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="74"/>
@@ -18689,25 +18695,51 @@
         <v>OK</v>
       </c>
     </row>
+    <row r="13" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="89" t="s">
+        <v>560</v>
+      </c>
+      <c r="B13" s="91" t="n">
+        <f aca="false">SUMPRODUCT(--ISNUMBER(Assumptions!$B$5:$B$42))</f>
+        <v>25</v>
+      </c>
+      <c r="C13" s="42" t="str">
+        <f aca="false">IF(B13=25,"OK","CHECK: fix the yellow/blue inputs")</f>
+        <v>OK</v>
+      </c>
+    </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="83" t="s">
+      <c r="A14" s="89" t="s">
+        <v>561</v>
+      </c>
+      <c r="B14" s="91" t="n">
+        <f aca="false">SUMPRODUCT(--ISERROR(Variables!$A$4:$G$80))</f>
+        <v>0</v>
+      </c>
+      <c r="C14" s="42" t="str">
+        <f aca="false">IF(B14=0,"OK","CHECK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="83" t="s">
         <v>46</v>
       </c>
-      <c r="C14" s="17" t="str">
-        <f aca="false">IF(COUNTIF(C5:C12,"OK")=8,"ALL OK","CHECK")</f>
+      <c r="C16" s="17" t="str">
+        <f aca="false">IF(COUNTIF(C5:C14,"OK")=10,"ALL OK","CHECK")</f>
         <v>ALL OK</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="53.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="49" t="s">
-        <v>560</v>
-      </c>
-      <c r="B15" s="49"/>
-      <c r="C15" s="49"/>
+    <row r="17" customFormat="false" ht="53.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="49" t="s">
+        <v>562</v>
+      </c>
+      <c r="B17" s="49"/>
+      <c r="C17" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A17:C17"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -19386,6 +19418,12 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation allowBlank="false" error="Type one plain number, e.g. 12 (not &quot;12-15&quot; or &quot;12 min&quot;). Ranges have separate low and high rows." errorStyle="stop" errorTitle="Numbers only" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B6:B10 B13:B15 B18:B21 B24:B28 B31:B32 B35:B38 B41:B42" type="decimal">
+      <formula1>0</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>